<commit_message>
CI Reports [2026-07-01 18:53]: AddNewUser — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
+++ b/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
@@ -505,10 +505,10 @@
         <v>h1='User Management'; addBtn visible; grid with user rows; stat cards shown</v>
       </c>
       <c r="K2" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L2" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M2" t="str">
         <v>Playwright Automation</v>
@@ -560,7 +560,7 @@
         <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
       </c>
       <c r="K3" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L3" t="str">
         <v>FAIL</v>
@@ -614,7 +614,7 @@
         <v>Success feedback; Partner User created</v>
       </c>
       <c r="K4" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L4" t="str">
         <v>FAIL</v>
@@ -669,7 +669,7 @@
         <v>Password input visible when Manual selected; user created successfully</v>
       </c>
       <c r="K5" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[name="passType"]').nth(1) - locator resolved to &lt;input type="radio" value="manual" name="passType" onchange="togglePassEntry()"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and</v>
       </c>
       <c r="L5" t="str">
         <v>FAIL</v>
@@ -722,7 +722,7 @@
         <v>User created with Inactive status; success feedback shown</v>
       </c>
       <c r="K6" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#fStatusInactive') - locator resolved to &lt;input type="radio" name="fStatus" value="inactive" id="fStatusInactive"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and stable - element is</v>
       </c>
       <c r="L6" t="str">
         <v>FAIL</v>
@@ -775,10 +775,10 @@
         <v>Modal closes; filled data discarded; no user created</v>
       </c>
       <c r="K7" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L7" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M7" t="str">
         <v>Playwright Automation</v>
@@ -828,10 +828,10 @@
         <v>Modal closes; no user created; data discarded</v>
       </c>
       <c r="K8" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L8" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M8" t="str">
         <v>Playwright Automation</v>
@@ -881,7 +881,7 @@
         <v>1-char First Name accepted; user created successfully</v>
       </c>
       <c r="K9" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L9" t="str">
         <v>FAIL</v>
@@ -933,7 +933,7 @@
         <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
       </c>
       <c r="K10" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L10" t="str">
         <v>FAIL</v>
@@ -985,7 +985,7 @@
         <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
       </c>
       <c r="K11" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L11" t="str">
         <v>FAIL</v>
@@ -1038,7 +1038,7 @@
         <v>"A valid email address is required" error; modal stays open</v>
       </c>
       <c r="K12" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L12" t="str">
         <v>FAIL</v>
@@ -1092,7 +1092,7 @@
         <v>"Please select a customer" shown; modal stays open</v>
       </c>
       <c r="K13" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L13" t="str">
         <v>FAIL</v>
@@ -1148,7 +1148,7 @@
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
       <c r="K14" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L14" t="str">
         <v>FAIL</v>
@@ -1255,7 +1255,7 @@
         <v>XSS payload not executed; alertFired=false; no script injection</v>
       </c>
       <c r="K16" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="L16" t="str">
         <v>FAIL</v>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P12"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -1357,13 +1357,13 @@
         <v>BUG-ADDNEWUSER-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Page loads with heading, stats, grid, Add New User button</v>
+        <v>Create Partner Admin — Automatic password</v>
       </c>
       <c r="C2" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D2" t="str">
-        <v>TC-AU-007</v>
+        <v>TC-AU-001</v>
       </c>
       <c r="E2" t="str">
         <v>Critical</v>
@@ -1375,67 +1375,68 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to page
-2. Check h1, button, grid presence</v>
-      </c>
-      <c r="I2" t="str">
-        <v>h1='User Management'; addBtn visible; grid with user rows; stat cards shown</v>
-      </c>
-      <c r="J2" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K2" t="str">
-        <v>New</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M2" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
-        <v>BUG-ADDNEWUSER-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Create Partner Admin — Automatic password</v>
-      </c>
-      <c r="C3" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D3" t="str">
-        <v>TC-AU-001</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Critical</v>
-      </c>
-      <c r="F3" t="str">
-        <v>P1</v>
-      </c>
-      <c r="G3" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open Add New User
 2. Fill all fields for Partner Admin
 3. Click Create User
 4. Check success feedback</v>
       </c>
+      <c r="I2" t="str">
+        <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
+      </c>
+      <c r="J2" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+      </c>
+      <c r="K2" t="str">
+        <v>New</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M2" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>Not Run</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>BUG-ADDNEWUSER-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Create Partner User — Automatic password</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-AU-002</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="H3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open modal
+2. Select Partner User role
+3. Check if Customer field is shown</v>
+      </c>
       <c r="I3" t="str">
-        <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
+        <v>Success feedback; Partner User created</v>
       </c>
       <c r="J3" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="K3" t="str">
         <v>New</v>
@@ -1461,13 +1462,13 @@
         <v>BUG-ADDNEWUSER-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Create Partner User — Automatic password</v>
+        <v>Create user with Manual password</v>
       </c>
       <c r="C4" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D4" t="str">
-        <v>TC-AU-002</v>
+        <v>TC-AU-003</v>
       </c>
       <c r="E4" t="str">
         <v>Low</v>
@@ -1479,15 +1480,15 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open modal
-2. Select Partner User role
-3. Check if Customer field is shown</v>
+        <v xml:space="preserve">1. Click Manual radio
+2. Check #fPassword visibility
+3. Fill and submit</v>
       </c>
       <c r="I4" t="str">
-        <v>Success feedback; Partner User created</v>
+        <v>Password input visible when Manual selected; user created successfully</v>
       </c>
       <c r="J4" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[name="passType"]').nth(1) - locator resolved to &lt;input type="radio" value="manual" name="passType" onchange="togglePassEntry()"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and</v>
       </c>
       <c r="K4" t="str">
         <v>New</v>
@@ -1513,13 +1514,13 @@
         <v>BUG-ADDNEWUSER-004</v>
       </c>
       <c r="B5" t="str">
-        <v>Create user with Manual password</v>
+        <v>Create user with Inactive status</v>
       </c>
       <c r="C5" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D5" t="str">
-        <v>TC-AU-003</v>
+        <v>TC-AU-005</v>
       </c>
       <c r="E5" t="str">
         <v>Low</v>
@@ -1531,15 +1532,15 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click Manual radio
-2. Check #fPassword visibility
-3. Fill and submit</v>
+        <v xml:space="preserve">1. Select Inactive
+2. Submit
+3. Confirm status</v>
       </c>
       <c r="I5" t="str">
-        <v>Password input visible when Manual selected; user created successfully</v>
+        <v>User created with Inactive status; success feedback shown</v>
       </c>
       <c r="J5" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#fStatusInactive') - locator resolved to &lt;input type="radio" name="fStatus" value="inactive" id="fStatusInactive"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and stable - element is</v>
       </c>
       <c r="K5" t="str">
         <v>New</v>
@@ -1565,16 +1566,16 @@
         <v>BUG-ADDNEWUSER-005</v>
       </c>
       <c r="B6" t="str">
-        <v>Create user with Inactive status</v>
+        <v>Single character First Name (min boundary) accepted</v>
       </c>
       <c r="C6" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D6" t="str">
-        <v>TC-AU-005</v>
+        <v>TC-AU-019</v>
       </c>
       <c r="E6" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="F6" t="str">
         <v>P3</v>
@@ -1583,15 +1584,15 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Select Inactive
+        <v xml:space="preserve">1. Enter "A" as First Name
 2. Submit
-3. Confirm status</v>
+3. Check if accepted</v>
       </c>
       <c r="I6" t="str">
-        <v>User created with Inactive status; success feedback shown</v>
+        <v>1-char First Name accepted; user created successfully</v>
       </c>
       <c r="J6" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="K6" t="str">
         <v>New</v>
@@ -1617,33 +1618,33 @@
         <v>BUG-ADDNEWUSER-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Cancel button closes modal without saving</v>
+        <v>Empty form submit shows all validation errors</v>
       </c>
       <c r="C7" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D7" t="str">
-        <v>TC-AU-008</v>
+        <v>TC-AU-013</v>
       </c>
       <c r="E7" t="str">
-        <v>Low</v>
+        <v>High</v>
       </c>
       <c r="F7" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="G7" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Fill some data
-2. Click Cancel
-3. Check modal state</v>
+        <v xml:space="preserve">1. Open modal
+2. Click Create User immediately
+3. Check all error messages</v>
       </c>
       <c r="I7" t="str">
-        <v>Modal closes; filled data discarded; no user created</v>
+        <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
       </c>
       <c r="J7" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="K7" t="str">
         <v>New</v>
@@ -1669,33 +1670,33 @@
         <v>BUG-ADDNEWUSER-007</v>
       </c>
       <c r="B8" t="str">
-        <v>Close (✕) button dismisses modal</v>
+        <v>Empty First Name shows validation error</v>
       </c>
       <c r="C8" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D8" t="str">
-        <v>TC-AU-006</v>
+        <v>TC-AU-010</v>
       </c>
       <c r="E8" t="str">
-        <v>Low</v>
+        <v>High</v>
       </c>
       <c r="F8" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="G8" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Fill partial data
-2. Click ✕
-3. Check if modal closed</v>
+        <v xml:space="preserve">1. Leave First Name empty
+2. Submit
+3. Check wrapFirstName error</v>
       </c>
       <c r="I8" t="str">
-        <v>Modal closes; no user created; data discarded</v>
+        <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
       </c>
       <c r="J8" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="K8" t="str">
         <v>New</v>
@@ -1721,33 +1722,33 @@
         <v>BUG-ADDNEWUSER-008</v>
       </c>
       <c r="B9" t="str">
-        <v>Single character First Name (min boundary) accepted</v>
+        <v>Invalid email format shows validation error</v>
       </c>
       <c r="C9" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D9" t="str">
-        <v>TC-AU-019</v>
+        <v>TC-AU-017</v>
       </c>
       <c r="E9" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="F9" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="G9" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Enter "A" as First Name
+        <v xml:space="preserve">1. Enter invalid email
 2. Submit
-3. Check if accepted</v>
+3. Check email error message</v>
       </c>
       <c r="I9" t="str">
-        <v>1-char First Name accepted; user created successfully</v>
+        <v>"A valid email address is required" error; modal stays open</v>
       </c>
       <c r="J9" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
       </c>
       <c r="K9" t="str">
         <v>New</v>
@@ -1773,317 +1774,161 @@
         <v>BUG-ADDNEWUSER-009</v>
       </c>
       <c r="B10" t="str">
-        <v>Empty form submit shows all validation errors</v>
+        <v>Partner User without customer shows validation error</v>
       </c>
       <c r="C10" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D10" t="str">
-        <v>TC-AU-013</v>
+        <v>TC-AU-018</v>
       </c>
       <c r="E10" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="F10" t="str">
-        <v>P2</v>
+        <v>P3</v>
       </c>
       <c r="G10" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open modal
-2. Click Create User immediately
-3. Check all error messages</v>
-      </c>
-      <c r="I10" t="str">
-        <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
-      </c>
-      <c r="J10" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K10" t="str">
-        <v>New</v>
-      </c>
-      <c r="L10" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M10" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N10" t="str">
-        <v/>
-      </c>
-      <c r="O10" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
-        <v>BUG-ADDNEWUSER-010</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Empty First Name shows validation error</v>
-      </c>
-      <c r="C11" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D11" t="str">
-        <v>TC-AU-010</v>
-      </c>
-      <c r="E11" t="str">
-        <v>High</v>
-      </c>
-      <c r="F11" t="str">
-        <v>P2</v>
-      </c>
-      <c r="G11" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H11" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Leave First Name empty
-2. Submit
-3. Check wrapFirstName error</v>
-      </c>
-      <c r="I11" t="str">
-        <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
-      </c>
-      <c r="J11" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K11" t="str">
-        <v>New</v>
-      </c>
-      <c r="L11" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M11" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N11" t="str">
-        <v/>
-      </c>
-      <c r="O11" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12" t="str">
-        <v>BUG-ADDNEWUSER-011</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Invalid email format shows validation error</v>
-      </c>
-      <c r="C12" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D12" t="str">
-        <v>TC-AU-017</v>
-      </c>
-      <c r="E12" t="str">
-        <v>High</v>
-      </c>
-      <c r="F12" t="str">
-        <v>P2</v>
-      </c>
-      <c r="G12" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H12" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Enter invalid email
-2. Submit
-3. Check email error message</v>
-      </c>
-      <c r="I12" t="str">
-        <v>"A valid email address is required" error; modal stays open</v>
-      </c>
-      <c r="J12" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K12" t="str">
-        <v>New</v>
-      </c>
-      <c r="L12" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M12" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N12" t="str">
-        <v/>
-      </c>
-      <c r="O12" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
-      <c r="A13" t="str">
-        <v>BUG-ADDNEWUSER-012</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Partner User without customer shows validation error</v>
-      </c>
-      <c r="C13" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D13" t="str">
-        <v>TC-AU-018</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F13" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G13" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select Partner User role
 2. Leave Customer empty
 3. Submit
 4. Check customer error</v>
       </c>
-      <c r="I13" t="str">
+      <c r="I10" t="str">
         <v>"Please select a customer" shown; modal stays open</v>
       </c>
-      <c r="J13" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K13" t="str">
+      <c r="J10" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+      </c>
+      <c r="K10" t="str">
         <v>New</v>
       </c>
-      <c r="L13" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M13" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N13" t="str">
-        <v/>
-      </c>
-      <c r="O13" t="str">
+      <c r="L10" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M10" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
-      <c r="A14" t="str">
-        <v>BUG-ADDNEWUSER-013</v>
-      </c>
-      <c r="B14" t="str">
+      <c r="P10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>BUG-ADDNEWUSER-010</v>
+      </c>
+      <c r="B11" t="str">
         <v>Duplicate username — silent failure BUG-AU-001</v>
       </c>
-      <c r="C14" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D14" t="str">
+      <c r="C11" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="D11" t="str">
         <v>TC-AU-015</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E11" t="str">
         <v>Critical</v>
       </c>
-      <c r="F14" t="str">
+      <c r="F11" t="str">
         <v>P1</v>
       </c>
-      <c r="G14" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H14" t="str" xml:space="preserve">
+      <c r="G11" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="H11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter existing username
 2. Submit
 3. Look for duplicate error message — currently none shown (BUG-AU-001)</v>
       </c>
-      <c r="I14" t="str">
+      <c r="I11" t="str">
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
-      <c r="J14" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K14" t="str">
+      <c r="J11" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+      </c>
+      <c r="K11" t="str">
         <v>New</v>
       </c>
-      <c r="L14" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M14" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N14" t="str">
-        <v/>
-      </c>
-      <c r="O14" t="str">
+      <c r="L11" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M11" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str">
-        <v>BUG-ADDNEWUSER-014</v>
-      </c>
-      <c r="B15" t="str">
+      <c r="P11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>BUG-ADDNEWUSER-011</v>
+      </c>
+      <c r="B12" t="str">
         <v>XSS payload in First Name does not execute</v>
       </c>
-      <c r="C15" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D15" t="str">
+      <c r="C12" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="D12" t="str">
         <v>TC-AU-021</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E12" t="str">
         <v>High</v>
       </c>
-      <c r="F15" t="str">
+      <c r="F12" t="str">
         <v>P2</v>
       </c>
-      <c r="G15" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H15" t="str" xml:space="preserve">
+      <c r="G12" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="H12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter XSS in First Name
 2. Submit
 3. Check if alert fires</v>
       </c>
-      <c r="I15" t="str">
+      <c r="I12" t="str">
         <v>XSS payload not executed; alertFired=false; no script injection</v>
       </c>
-      <c r="J15" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K15" t="str">
+      <c r="J12" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+      </c>
+      <c r="K12" t="str">
         <v>New</v>
       </c>
-      <c r="L15" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M15" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N15" t="str">
-        <v/>
-      </c>
-      <c r="O15" t="str">
+      <c r="L12" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M12" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P15" t="str">
+      <c r="P12" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 19:07]: AddNewUser — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
+++ b/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
@@ -560,7 +560,7 @@
         <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
       </c>
       <c r="K3" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="L3" t="str">
         <v>FAIL</v>
@@ -614,7 +614,7 @@
         <v>Success feedback; Partner User created</v>
       </c>
       <c r="K4" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="L4" t="str">
         <v>FAIL</v>
@@ -669,7 +669,7 @@
         <v>Password input visible when Manual selected; user created successfully</v>
       </c>
       <c r="K5" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[name="passType"]').nth(1) - locator resolved to &lt;input type="radio" value="manual" name="passType" onchange="togglePassEntry()"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="L5" t="str">
         <v>FAIL</v>
@@ -722,7 +722,7 @@
         <v>User created with Inactive status; success feedback shown</v>
       </c>
       <c r="K6" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#fStatusInactive') - locator resolved to &lt;input type="radio" name="fStatus" value="inactive" id="fStatusInactive"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and stable - element is</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="L6" t="str">
         <v>FAIL</v>
@@ -881,7 +881,7 @@
         <v>1-char First Name accepted; user created successfully</v>
       </c>
       <c r="K9" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="L9" t="str">
         <v>FAIL</v>
@@ -933,10 +933,10 @@
         <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
       </c>
       <c r="K10" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L10" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M10" t="str">
         <v>Playwright Automation</v>
@@ -985,10 +985,10 @@
         <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
       </c>
       <c r="K11" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L11" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M11" t="str">
         <v>Playwright Automation</v>
@@ -1038,10 +1038,10 @@
         <v>"A valid email address is required" error; modal stays open</v>
       </c>
       <c r="K12" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L12" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M12" t="str">
         <v>Playwright Automation</v>
@@ -1092,7 +1092,7 @@
         <v>"Please select a customer" shown; modal stays open</v>
       </c>
       <c r="K13" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(locator).toHaveText(expected) failed Locator: locator('#wrapCustomer .um-field-error') Expected: "Please select a customer" Received: "Select at least one customer" Timeout: 5000ms Call log: - Expect "toHaveText" with timeout 5000ms - waiting for locator('#wrapCustomer .um-field-error'</v>
       </c>
       <c r="L13" t="str">
         <v>FAIL</v>
@@ -1148,7 +1148,7 @@
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
       <c r="K14" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#wrapUsername .um-field-error') Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#wrapUsername .um-field-error') 14 × locator resolved to &lt;div class="um-field-e</v>
       </c>
       <c r="L14" t="str">
         <v>FAIL</v>
@@ -1255,10 +1255,10 @@
         <v>XSS payload not executed; alertFired=false; no script injection</v>
       </c>
       <c r="K16" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L16" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M16" t="str">
         <v>Playwright Automation</v>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P8"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -1384,7 +1384,7 @@
         <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
       </c>
       <c r="J2" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K2" t="str">
         <v>New</v>
@@ -1436,7 +1436,7 @@
         <v>Success feedback; Partner User created</v>
       </c>
       <c r="J3" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K3" t="str">
         <v>New</v>
@@ -1488,7 +1488,7 @@
         <v>Password input visible when Manual selected; user created successfully</v>
       </c>
       <c r="J4" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[name="passType"]').nth(1) - locator resolved to &lt;input type="radio" value="manual" name="passType" onchange="togglePassEntry()"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K4" t="str">
         <v>New</v>
@@ -1540,7 +1540,7 @@
         <v>User created with Inactive status; success feedback shown</v>
       </c>
       <c r="J5" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#fStatusInactive') - locator resolved to &lt;input type="radio" name="fStatus" value="inactive" id="fStatusInactive"/&gt; - attempting click action 2 × waiting for element to be visible, enabled and stable - element is</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K5" t="str">
         <v>New</v>
@@ -1592,7 +1592,7 @@
         <v>1-char First Name accepted; user created successfully</v>
       </c>
       <c r="J6" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
+        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
       </c>
       <c r="K6" t="str">
         <v>New</v>
@@ -1618,317 +1618,109 @@
         <v>BUG-ADDNEWUSER-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Empty form submit shows all validation errors</v>
+        <v>Partner User without customer shows validation error</v>
       </c>
       <c r="C7" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D7" t="str">
-        <v>TC-AU-013</v>
+        <v>TC-AU-018</v>
       </c>
       <c r="E7" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="F7" t="str">
-        <v>P2</v>
+        <v>P3</v>
       </c>
       <c r="G7" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open modal
-2. Click Create User immediately
-3. Check all error messages</v>
-      </c>
-      <c r="I7" t="str">
-        <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
-      </c>
-      <c r="J7" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K7" t="str">
-        <v>New</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M7" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N7" t="str">
-        <v/>
-      </c>
-      <c r="O7" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>BUG-ADDNEWUSER-007</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Empty First Name shows validation error</v>
-      </c>
-      <c r="C8" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D8" t="str">
-        <v>TC-AU-010</v>
-      </c>
-      <c r="E8" t="str">
-        <v>High</v>
-      </c>
-      <c r="F8" t="str">
-        <v>P2</v>
-      </c>
-      <c r="G8" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Leave First Name empty
-2. Submit
-3. Check wrapFirstName error</v>
-      </c>
-      <c r="I8" t="str">
-        <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
-      </c>
-      <c r="J8" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K8" t="str">
-        <v>New</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M8" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N8" t="str">
-        <v/>
-      </c>
-      <c r="O8" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str">
-        <v>BUG-ADDNEWUSER-008</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Invalid email format shows validation error</v>
-      </c>
-      <c r="C9" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D9" t="str">
-        <v>TC-AU-017</v>
-      </c>
-      <c r="E9" t="str">
-        <v>High</v>
-      </c>
-      <c r="F9" t="str">
-        <v>P2</v>
-      </c>
-      <c r="G9" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Enter invalid email
-2. Submit
-3. Check email error message</v>
-      </c>
-      <c r="I9" t="str">
-        <v>"A valid email address is required" error; modal stays open</v>
-      </c>
-      <c r="J9" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K9" t="str">
-        <v>New</v>
-      </c>
-      <c r="L9" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M9" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N9" t="str">
-        <v/>
-      </c>
-      <c r="O9" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
-        <v>BUG-ADDNEWUSER-009</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Partner User without customer shows validation error</v>
-      </c>
-      <c r="C10" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D10" t="str">
-        <v>TC-AU-018</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F10" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G10" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select Partner User role
 2. Leave Customer empty
 3. Submit
 4. Check customer error</v>
       </c>
-      <c r="I10" t="str">
+      <c r="I7" t="str">
         <v>"Please select a customer" shown; modal stays open</v>
       </c>
-      <c r="J10" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K10" t="str">
+      <c r="J7" t="str">
+        <v>Error: expect(locator).toHaveText(expected) failed Locator: locator('#wrapCustomer .um-field-error') Expected: "Please select a customer" Received: "Select at least one customer" Timeout: 5000ms Call log: - Expect "toHaveText" with timeout 5000ms - waiting for locator('#wrapCustomer .um-field-error'</v>
+      </c>
+      <c r="K7" t="str">
         <v>New</v>
       </c>
-      <c r="L10" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M10" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N10" t="str">
-        <v/>
-      </c>
-      <c r="O10" t="str">
+      <c r="L7" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M7" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
-        <v>BUG-ADDNEWUSER-010</v>
-      </c>
-      <c r="B11" t="str">
+      <c r="P7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>BUG-ADDNEWUSER-007</v>
+      </c>
+      <c r="B8" t="str">
         <v>Duplicate username — silent failure BUG-AU-001</v>
       </c>
-      <c r="C11" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D11" t="str">
+      <c r="C8" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="D8" t="str">
         <v>TC-AU-015</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E8" t="str">
         <v>Critical</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F8" t="str">
         <v>P1</v>
       </c>
-      <c r="G11" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H11" t="str" xml:space="preserve">
+      <c r="G8" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
+      </c>
+      <c r="H8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter existing username
 2. Submit
 3. Look for duplicate error message — currently none shown (BUG-AU-001)</v>
       </c>
-      <c r="I11" t="str">
+      <c r="I8" t="str">
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
-      <c r="J11" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K11" t="str">
+      <c r="J8" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#wrapUsername .um-field-error') Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#wrapUsername .um-field-error') 14 × locator resolved to &lt;div class="um-field-e</v>
+      </c>
+      <c r="K8" t="str">
         <v>New</v>
       </c>
-      <c r="L11" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M11" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N11" t="str">
-        <v/>
-      </c>
-      <c r="O11" t="str">
+      <c r="L8" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M8" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12" t="str">
-        <v>BUG-ADDNEWUSER-011</v>
-      </c>
-      <c r="B12" t="str">
-        <v>XSS payload in First Name does not execute</v>
-      </c>
-      <c r="C12" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D12" t="str">
-        <v>TC-AU-021</v>
-      </c>
-      <c r="E12" t="str">
-        <v>High</v>
-      </c>
-      <c r="F12" t="str">
-        <v>P2</v>
-      </c>
-      <c r="G12" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H12" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Enter XSS in First Name
-2. Submit
-3. Check if alert fires</v>
-      </c>
-      <c r="I12" t="str">
-        <v>XSS payload not executed; alertFired=false; no script injection</v>
-      </c>
-      <c r="J12" t="str">
-        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('button.um-btn-primary').last() - locator resolved to &lt;button id="feedbackCloseBtn" class="um-btn-primary" onclick="closeFeedbackModal()"&gt;…&lt;/button&gt; - attempting click action 2 × waiting for element to be visible,</v>
-      </c>
-      <c r="K12" t="str">
-        <v>New</v>
-      </c>
-      <c r="L12" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M12" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N12" t="str">
-        <v/>
-      </c>
-      <c r="O12" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P12" t="str">
+      <c r="P8" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 19:17]: AddNewUser — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
+++ b/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
@@ -1092,10 +1092,10 @@
         <v>"Please select a customer" shown; modal stays open</v>
       </c>
       <c r="K13" t="str">
-        <v>Error: expect(locator).toHaveText(expected) failed Locator: locator('#wrapCustomer .um-field-error') Expected: "Please select a customer" Received: "Select at least one customer" Timeout: 5000ms Call log: - Expect "toHaveText" with timeout 5000ms - waiting for locator('#wrapCustomer .um-field-error'</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L13" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M13" t="str">
         <v>Playwright Automation</v>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -1618,109 +1618,56 @@
         <v>BUG-ADDNEWUSER-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Partner User without customer shows validation error</v>
+        <v>Duplicate username — silent failure BUG-AU-001</v>
       </c>
       <c r="C7" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D7" t="str">
-        <v>TC-AU-018</v>
+        <v>TC-AU-015</v>
       </c>
       <c r="E7" t="str">
-        <v>Low</v>
+        <v>Critical</v>
       </c>
       <c r="F7" t="str">
-        <v>P3</v>
+        <v>P1</v>
       </c>
       <c r="G7" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Select Partner User role
-2. Leave Customer empty
-3. Submit
-4. Check customer error</v>
-      </c>
-      <c r="I7" t="str">
-        <v>"Please select a customer" shown; modal stays open</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Error: expect(locator).toHaveText(expected) failed Locator: locator('#wrapCustomer .um-field-error') Expected: "Please select a customer" Received: "Select at least one customer" Timeout: 5000ms Call log: - Expect "toHaveText" with timeout 5000ms - waiting for locator('#wrapCustomer .um-field-error'</v>
-      </c>
-      <c r="K7" t="str">
-        <v>New</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M7" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N7" t="str">
-        <v/>
-      </c>
-      <c r="O7" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>BUG-ADDNEWUSER-007</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Duplicate username — silent failure BUG-AU-001</v>
-      </c>
-      <c r="C8" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D8" t="str">
-        <v>TC-AU-015</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Critical</v>
-      </c>
-      <c r="F8" t="str">
-        <v>P1</v>
-      </c>
-      <c r="G8" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter existing username
 2. Submit
 3. Look for duplicate error message — currently none shown (BUG-AU-001)</v>
       </c>
-      <c r="I8" t="str">
+      <c r="I7" t="str">
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J7" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('#wrapUsername .um-field-error') Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#wrapUsername .um-field-error') 14 × locator resolved to &lt;div class="um-field-e</v>
       </c>
-      <c r="K8" t="str">
+      <c r="K7" t="str">
         <v>New</v>
       </c>
-      <c r="L8" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M8" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N8" t="str">
-        <v/>
-      </c>
-      <c r="O8" t="str">
+      <c r="L7" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M7" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P8" t="str">
+      <c r="P7" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 20:24]: AddNewUser — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
+++ b/Test Execution Report_Git/Feature Reports/AddNewUser.xlsx
@@ -560,10 +560,10 @@
         <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
       </c>
       <c r="K3" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L3" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M3" t="str">
         <v>Playwright Automation</v>
@@ -614,10 +614,10 @@
         <v>Success feedback; Partner User created</v>
       </c>
       <c r="K4" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L4" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M4" t="str">
         <v>Playwright Automation</v>
@@ -669,10 +669,10 @@
         <v>Password input visible when Manual selected; user created successfully</v>
       </c>
       <c r="K5" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L5" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M5" t="str">
         <v>Playwright Automation</v>
@@ -722,10 +722,10 @@
         <v>User created with Inactive status; success feedback shown</v>
       </c>
       <c r="K6" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L6" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M6" t="str">
         <v>Playwright Automation</v>
@@ -881,10 +881,10 @@
         <v>1-char First Name accepted; user created successfully</v>
       </c>
       <c r="K9" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L9" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M9" t="str">
         <v>Playwright Automation</v>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -1357,13 +1357,13 @@
         <v>BUG-ADDNEWUSER-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Create Partner Admin — Automatic password</v>
+        <v>Duplicate username — silent failure BUG-AU-001</v>
       </c>
       <c r="C2" t="str">
         <v>AddNewUser</v>
       </c>
       <c r="D2" t="str">
-        <v>TC-AU-001</v>
+        <v>TC-AU-015</v>
       </c>
       <c r="E2" t="str">
         <v>Critical</v>
@@ -1375,299 +1375,38 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open Add New User
-2. Fill all fields for Partner Admin
-3. Click Create User
-4. Check success feedback</v>
-      </c>
-      <c r="I2" t="str">
-        <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
-      </c>
-      <c r="K2" t="str">
-        <v>New</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M2" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
-        <v>BUG-ADDNEWUSER-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Create Partner User — Automatic password</v>
-      </c>
-      <c r="C3" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D3" t="str">
-        <v>TC-AU-002</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F3" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G3" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open modal
-2. Select Partner User role
-3. Check if Customer field is shown</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Success feedback; Partner User created</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
-      </c>
-      <c r="K3" t="str">
-        <v>New</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M3" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>BUG-ADDNEWUSER-003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Create user with Manual password</v>
-      </c>
-      <c r="C4" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D4" t="str">
-        <v>TC-AU-003</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F4" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G4" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click Manual radio
-2. Check #fPassword visibility
-3. Fill and submit</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Password input visible when Manual selected; user created successfully</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
-      </c>
-      <c r="K4" t="str">
-        <v>New</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M4" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>BUG-ADDNEWUSER-004</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Create user with Inactive status</v>
-      </c>
-      <c r="C5" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D5" t="str">
-        <v>TC-AU-005</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F5" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G5" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Select Inactive
-2. Submit
-3. Confirm status</v>
-      </c>
-      <c r="I5" t="str">
-        <v>User created with Inactive status; success feedback shown</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
-      </c>
-      <c r="K5" t="str">
-        <v>New</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M5" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N5" t="str">
-        <v/>
-      </c>
-      <c r="O5" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>BUG-ADDNEWUSER-005</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Single character First Name (min boundary) accepted</v>
-      </c>
-      <c r="C6" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D6" t="str">
-        <v>TC-AU-019</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="F6" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G6" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Enter "A" as First Name
-2. Submit
-3. Check if accepted</v>
-      </c>
-      <c r="I6" t="str">
-        <v>1-char First Name accepted; user created successfully</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Error: expect(received).toBe(expected) // Object.is equality Expected: true Received: false</v>
-      </c>
-      <c r="K6" t="str">
-        <v>New</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M6" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N6" t="str">
-        <v/>
-      </c>
-      <c r="O6" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
-        <v>BUG-ADDNEWUSER-006</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Duplicate username — silent failure BUG-AU-001</v>
-      </c>
-      <c r="C7" t="str">
-        <v>AddNewUser</v>
-      </c>
-      <c r="D7" t="str">
-        <v>TC-AU-015</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Critical</v>
-      </c>
-      <c r="F7" t="str">
-        <v>P1</v>
-      </c>
-      <c r="G7" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter existing username
 2. Submit
 3. Look for duplicate error message — currently none shown (BUG-AU-001)</v>
       </c>
-      <c r="I7" t="str">
+      <c r="I2" t="str">
         <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J2" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('#wrapUsername .um-field-error') Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#wrapUsername .um-field-error') 14 × locator resolved to &lt;div class="um-field-e</v>
       </c>
-      <c r="K7" t="str">
+      <c r="K2" t="str">
         <v>New</v>
       </c>
-      <c r="L7" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M7" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N7" t="str">
-        <v/>
-      </c>
-      <c r="O7" t="str">
+      <c r="L2" t="str">
+        <v>Playwright Automation</v>
+      </c>
+      <c r="M2" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>Not Run</v>
       </c>
-      <c r="P7" t="str">
+      <c r="P2" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>